<commit_message>
Enhance missing payment handling with improved record counting and UI updates
</commit_message>
<xml_diff>
--- a/assets/template/Missing Pament Details.xlsx
+++ b/assets/template/Missing Pament Details.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t xml:space="preserve">Coustomer ID</t>
   </si>
@@ -52,6 +52,9 @@
   </si>
   <si>
     <t xml:space="preserve">Missing fine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missing week</t>
   </si>
 </sst>
 </file>
@@ -189,11 +192,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -461,8 +464,9 @@
       <c r="B7" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="0"/>
+      <c r="C7" s="9" t="s">
+        <v>10</v>
+      </c>
       <c r="F7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -470,104 +474,114 @@
         <v>46254</v>
       </c>
       <c r="B8" s="11"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="0"/>
-      <c r="F8" s="13"/>
+      <c r="C8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="12"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="n">
         <v>46255</v>
       </c>
       <c r="B9" s="11"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="0"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
+      <c r="C9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="n">
         <v>46256</v>
       </c>
       <c r="B10" s="11"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="0"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
+      <c r="C10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="n">
         <v>46258</v>
       </c>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="0"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="n">
         <v>46259</v>
       </c>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="0"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="n">
         <v>46260</v>
       </c>
-      <c r="B13" s="12" t="n">
-        <v>15</v>
-      </c>
-      <c r="C13" s="12"/>
-      <c r="D13" s="0"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="13"/>
+      <c r="B13" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="13"/>
+      <c r="G13" s="12"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="n">
         <v>46261</v>
       </c>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="0"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="E14" s="7"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="12"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="n">
         <v>46262</v>
       </c>
-      <c r="B15" s="12"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="0"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="13"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="13"/>
+      <c r="G15" s="12"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="n">
         <v>46263</v>
       </c>
-      <c r="B16" s="12" t="n">
-        <v>15</v>
-      </c>
-      <c r="C16" s="12"/>
-      <c r="D16" s="0"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="13"/>
+      <c r="B16" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="13"/>
+      <c r="G16" s="12"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="n">
         <v>46265</v>
       </c>
       <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="0"/>
+      <c r="C17" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F17" s="14"/>
-      <c r="G17" s="13"/>
+      <c r="G17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="n">
@@ -576,41 +590,45 @@
       <c r="B18" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="0"/>
+      <c r="C18" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F18" s="14"/>
-      <c r="G18" s="13"/>
+      <c r="G18" s="12"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="n">
         <v>46268</v>
       </c>
       <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="0"/>
+      <c r="C19" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="E19" s="7"/>
       <c r="F19" s="14"/>
-      <c r="G19" s="13"/>
+      <c r="G19" s="12"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="n">
         <v>46269</v>
       </c>
       <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="0"/>
+      <c r="C20" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F20" s="14"/>
-      <c r="G20" s="13"/>
+      <c r="G20" s="12"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="n">
         <v>46270</v>
       </c>
       <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="0"/>
+      <c r="C21" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F21" s="14"/>
-      <c r="G21" s="13"/>
+      <c r="G21" s="12"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="n">
@@ -619,10 +637,11 @@
       <c r="B22" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C22" s="14"/>
-      <c r="D22" s="0"/>
+      <c r="C22" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F22" s="14"/>
-      <c r="G22" s="13"/>
+      <c r="G22" s="12"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="n">
@@ -631,40 +650,44 @@
       <c r="B23" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="0"/>
+      <c r="C23" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F23" s="14"/>
-      <c r="G23" s="13"/>
+      <c r="G23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="n">
         <v>46274</v>
       </c>
       <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="0"/>
+      <c r="C24" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F24" s="14"/>
-      <c r="G24" s="13"/>
+      <c r="G24" s="12"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="n">
         <v>46275</v>
       </c>
       <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="0"/>
+      <c r="C25" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F25" s="14"/>
-      <c r="G25" s="13"/>
+      <c r="G25" s="12"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="n">
         <v>46276</v>
       </c>
       <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="0"/>
+      <c r="C26" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F26" s="14"/>
-      <c r="G26" s="13"/>
+      <c r="G26" s="12"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="n">
@@ -673,20 +696,22 @@
       <c r="B27" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C27" s="14"/>
-      <c r="D27" s="0"/>
+      <c r="C27" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F27" s="14"/>
-      <c r="G27" s="13"/>
+      <c r="G27" s="12"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="n">
         <v>46279</v>
       </c>
       <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="0"/>
+      <c r="C28" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F28" s="14"/>
-      <c r="G28" s="13"/>
+      <c r="G28" s="12"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="n">
@@ -695,10 +720,11 @@
       <c r="B29" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C29" s="14"/>
-      <c r="D29" s="0"/>
+      <c r="C29" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F29" s="14"/>
-      <c r="G29" s="13"/>
+      <c r="G29" s="12"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="n">
@@ -707,10 +733,11 @@
       <c r="B30" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C30" s="14"/>
-      <c r="D30" s="0"/>
+      <c r="C30" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F30" s="14"/>
-      <c r="G30" s="13"/>
+      <c r="G30" s="12"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="n">
@@ -719,20 +746,22 @@
       <c r="B31" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C31" s="14"/>
-      <c r="D31" s="0"/>
+      <c r="C31" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F31" s="14"/>
-      <c r="G31" s="13"/>
+      <c r="G31" s="12"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="n">
         <v>46283</v>
       </c>
       <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="0"/>
+      <c r="C32" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F32" s="14"/>
-      <c r="G32" s="13"/>
+      <c r="G32" s="12"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="n">
@@ -741,10 +770,11 @@
       <c r="B33" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C33" s="14"/>
-      <c r="D33" s="0"/>
+      <c r="C33" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F33" s="14"/>
-      <c r="G33" s="13"/>
+      <c r="G33" s="12"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="n">
@@ -753,10 +783,11 @@
       <c r="B34" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C34" s="14"/>
-      <c r="D34" s="0"/>
+      <c r="C34" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F34" s="14"/>
-      <c r="G34" s="13"/>
+      <c r="G34" s="12"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="n">
@@ -765,10 +796,11 @@
       <c r="B35" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C35" s="14"/>
-      <c r="D35" s="0"/>
+      <c r="C35" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F35" s="14"/>
-      <c r="G35" s="13"/>
+      <c r="G35" s="12"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="n">
@@ -777,10 +809,11 @@
       <c r="B36" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C36" s="14"/>
-      <c r="D36" s="0"/>
+      <c r="C36" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F36" s="14"/>
-      <c r="G36" s="13"/>
+      <c r="G36" s="12"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="n">
@@ -789,10 +822,11 @@
       <c r="B37" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C37" s="14"/>
-      <c r="D37" s="0"/>
+      <c r="C37" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F37" s="14"/>
-      <c r="G37" s="13"/>
+      <c r="G37" s="12"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="n">
@@ -801,10 +835,11 @@
       <c r="B38" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C38" s="14"/>
-      <c r="D38" s="0"/>
+      <c r="C38" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F38" s="14"/>
-      <c r="G38" s="13"/>
+      <c r="G38" s="12"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="n">
@@ -813,13 +848,14 @@
       <c r="B39" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C39" s="14"/>
-      <c r="D39" s="0"/>
+      <c r="C39" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="F39" s="14"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10"/>
-      <c r="B40" s="12"/>
+      <c r="B40" s="13"/>
       <c r="C40" s="14"/>
       <c r="D40" s="14"/>
       <c r="F40" s="14"/>

</xml_diff>